<commit_message>
fix(map): map technical colleges strictly inside block polygons and enhance mobile responsiveness
</commit_message>
<xml_diff>
--- a/kanyakumari_colleges_verified_final.xlsx
+++ b/kanyakumari_colleges_verified_final.xlsx
@@ -10012,7 +10012,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O119" t="inlineStr"/>
       <c r="P119" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -10095,7 +10094,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O120" t="inlineStr"/>
       <c r="P120" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -10178,7 +10176,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O121" t="inlineStr"/>
       <c r="P121" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -10261,7 +10258,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O122" t="inlineStr"/>
       <c r="P122" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -10344,7 +10340,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O123" t="inlineStr"/>
       <c r="P123" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -10427,7 +10422,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O124" t="inlineStr"/>
       <c r="P124" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -10510,7 +10504,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O125" t="inlineStr"/>
       <c r="P125" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -10593,7 +10586,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O126" t="inlineStr"/>
       <c r="P126" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -10676,7 +10668,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O127" t="inlineStr"/>
       <c r="P127" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -10759,7 +10750,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O128" t="inlineStr"/>
       <c r="P128" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -10842,7 +10832,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O129" t="inlineStr"/>
       <c r="P129" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -10925,7 +10914,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O130" t="inlineStr"/>
       <c r="P130" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -11008,7 +10996,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O131" t="inlineStr"/>
       <c r="P131" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -11091,7 +11078,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O132" t="inlineStr"/>
       <c r="P132" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -11174,7 +11160,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O133" t="inlineStr"/>
       <c r="P133" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -11257,7 +11242,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O134" t="inlineStr"/>
       <c r="P134" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -11340,7 +11324,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O135" t="inlineStr"/>
       <c r="P135" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -11423,7 +11406,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O136" t="inlineStr"/>
       <c r="P136" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -11506,7 +11488,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O137" t="inlineStr"/>
       <c r="P137" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -11589,7 +11570,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O138" t="inlineStr"/>
       <c r="P138" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -11672,7 +11652,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O139" t="inlineStr"/>
       <c r="P139" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -11755,7 +11734,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O140" t="inlineStr"/>
       <c r="P140" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -11838,7 +11816,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O141" t="inlineStr"/>
       <c r="P141" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -11921,7 +11898,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O142" t="inlineStr"/>
       <c r="P142" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -12004,7 +11980,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O143" t="inlineStr"/>
       <c r="P143" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -12087,7 +12062,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O144" t="inlineStr"/>
       <c r="P144" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -12170,7 +12144,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O145" t="inlineStr"/>
       <c r="P145" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -12253,7 +12226,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O146" t="inlineStr"/>
       <c r="P146" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -12336,7 +12308,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O147" t="inlineStr"/>
       <c r="P147" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -12419,7 +12390,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O148" t="inlineStr"/>
       <c r="P148" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -12502,7 +12472,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O149" t="inlineStr"/>
       <c r="P149" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -12585,7 +12554,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O150" t="inlineStr"/>
       <c r="P150" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -12668,7 +12636,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O151" t="inlineStr"/>
       <c r="P151" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>
@@ -12751,7 +12718,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="O152" t="inlineStr"/>
       <c r="P152" t="inlineStr">
         <is>
           <t>Verified (TNDTE / NCVT MIS)</t>

</xml_diff>